<commit_message>
Updated System Interface Design
to include inputs and outputs relating to use case Grant Permission.
</commit_message>
<xml_diff>
--- a/Requester_and_Audio_Analyzer_System_Interface_Design.xlsx
+++ b/Requester_and_Audio_Analyzer_System_Interface_Design.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thoma\Documents\GitHub\Audio_Analyzer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F3ED78A-2630-40CA-9F2F-C527AFF5DC9D}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85C83EAD-4D28-4F3A-9536-9B579C8886D1}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19260" yWindow="50" windowWidth="19060" windowHeight="20670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19180" yWindow="0" windowWidth="19060" windowHeight="20670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="88">
   <si>
     <t>Name</t>
   </si>
@@ -281,6 +281,15 @@
   </si>
   <si>
     <t>Requested amalgamation</t>
+  </si>
+  <si>
+    <t>Grant Permission</t>
+  </si>
+  <si>
+    <t>Signal of desire to process audio files or listen to / view an amalgamation</t>
+  </si>
+  <si>
+    <t>Permission to process audio files or listen to / view an amalgamation</t>
   </si>
 </sst>
 </file>
@@ -359,7 +368,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -388,10 +397,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -680,7 +693,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:E71"/>
+  <dimension ref="A2:E73"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="28.26953125" bestFit="1" customWidth="1"/>
@@ -721,7 +734,7 @@
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="18" t="s">
         <v>59</v>
       </c>
       <c r="C10" s="15" t="s">
@@ -732,8 +745,8 @@
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B11" s="13"/>
-      <c r="C11" s="13" t="s">
+      <c r="B11" s="18"/>
+      <c r="C11" s="18" t="s">
         <v>47</v>
       </c>
       <c r="D11" s="6" t="s">
@@ -741,98 +754,98 @@
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B12" s="13"/>
-      <c r="C12" s="13"/>
+      <c r="B12" s="18"/>
+      <c r="C12" s="18"/>
       <c r="D12" s="6" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B13" s="13"/>
-      <c r="C13" s="13"/>
+      <c r="B13" s="18"/>
+      <c r="C13" s="18"/>
       <c r="D13" s="6" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B14" s="13"/>
-      <c r="C14" s="13"/>
+      <c r="B14" s="18"/>
+      <c r="C14" s="18"/>
       <c r="D14" s="7" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B15" s="13"/>
-      <c r="C15" s="14"/>
+      <c r="B15" s="18"/>
+      <c r="C15" s="19"/>
       <c r="D15" s="7" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B16" s="13"/>
-      <c r="C16" s="14"/>
+      <c r="B16" s="18"/>
+      <c r="C16" s="19"/>
       <c r="D16" s="7" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B17" s="13"/>
-      <c r="C17" s="14"/>
+      <c r="B17" s="18"/>
+      <c r="C17" s="19"/>
       <c r="D17" s="7" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B18" s="13"/>
-      <c r="C18" s="14"/>
+      <c r="B18" s="18"/>
+      <c r="C18" s="19"/>
       <c r="D18" s="7" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B19" s="13"/>
-      <c r="C19" s="14"/>
+      <c r="B19" s="18"/>
+      <c r="C19" s="19"/>
       <c r="D19" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B20" s="13"/>
-      <c r="C20" s="14"/>
+      <c r="B20" s="18"/>
+      <c r="C20" s="19"/>
       <c r="D20" s="7" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B21" s="13"/>
-      <c r="C21" s="14"/>
+      <c r="B21" s="18"/>
+      <c r="C21" s="19"/>
       <c r="D21" s="7" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B22" s="13"/>
-      <c r="C22" s="14"/>
+      <c r="B22" s="18"/>
+      <c r="C22" s="19"/>
       <c r="D22" s="8" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B23" s="13"/>
-      <c r="C23" s="14"/>
+      <c r="B23" s="18"/>
+      <c r="C23" s="19"/>
       <c r="D23" s="8" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B24" s="13"/>
-      <c r="C24" s="14"/>
+      <c r="B24" s="18"/>
+      <c r="C24" s="19"/>
       <c r="D24" s="8" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B25" s="13"/>
+      <c r="B25" s="18"/>
       <c r="C25" s="5" t="s">
         <v>48</v>
       </c>
@@ -841,7 +854,7 @@
       </c>
     </row>
     <row r="26" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B26" s="13"/>
+      <c r="B26" s="18"/>
       <c r="C26" s="5" t="s">
         <v>50</v>
       </c>
@@ -850,7 +863,7 @@
       </c>
     </row>
     <row r="27" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B27" s="13" t="s">
+      <c r="B27" s="18" t="s">
         <v>58</v>
       </c>
       <c r="C27" s="5" t="s">
@@ -861,7 +874,7 @@
       </c>
     </row>
     <row r="28" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B28" s="13"/>
+      <c r="B28" s="18"/>
       <c r="C28" s="5" t="s">
         <v>61</v>
       </c>
@@ -870,7 +883,7 @@
       </c>
     </row>
     <row r="29" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B29" s="13"/>
+      <c r="B29" s="18"/>
       <c r="C29" s="5" t="s">
         <v>62</v>
       </c>
@@ -879,7 +892,7 @@
       </c>
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B30" s="13"/>
+      <c r="B30" s="18"/>
       <c r="C30" s="5" t="s">
         <v>63</v>
       </c>
@@ -888,7 +901,7 @@
       </c>
     </row>
     <row r="31" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B31" t="s">
+      <c r="B31" s="18" t="s">
         <v>71</v>
       </c>
       <c r="C31" s="5" t="s">
@@ -899,6 +912,7 @@
       </c>
     </row>
     <row r="32" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B32" s="18"/>
       <c r="C32" s="5" t="s">
         <v>82</v>
       </c>
@@ -906,213 +920,214 @@
         <v>49</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A34" s="2" t="s">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B33" t="s">
+        <v>85</v>
+      </c>
+      <c r="C33" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="D33" s="16" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A35" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B35" s="3" t="s">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B36" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C35" s="3" t="s">
+      <c r="C36" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="D35" s="3" t="s">
+      <c r="D36" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B36" s="17" t="s">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B37" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="C36" s="15" t="s">
+      <c r="C37" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="D36" s="15" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B37" s="17"/>
-      <c r="C37" s="15" t="s">
+      <c r="D37" s="15" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B38" s="20"/>
+      <c r="C38" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="D37" s="15" t="s">
+      <c r="D38" s="15" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B38" s="17"/>
-      <c r="C38" s="15" t="s">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B39" s="20"/>
+      <c r="C39" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="D38" s="15" t="s">
+      <c r="D39" s="15" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B39" s="17"/>
-      <c r="C39" s="15" t="s">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B40" s="20"/>
+      <c r="C40" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="D39" s="15" t="s">
+      <c r="D40" s="15" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B40" s="17"/>
-      <c r="C40" s="13" t="s">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B41" s="20"/>
+      <c r="C41" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="D40" t="s">
+      <c r="D41" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B41" s="17"/>
-      <c r="C41" s="13"/>
-      <c r="D41" t="s">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B42" s="20"/>
+      <c r="C42" s="18"/>
+      <c r="D42" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B42" s="17"/>
-      <c r="C42" s="13"/>
-      <c r="D42" t="s">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B43" s="20"/>
+      <c r="C43" s="18"/>
+      <c r="D43" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B43" s="13" t="s">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B44" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="C43" s="4" t="s">
+      <c r="C44" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="D43" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B44" s="13"/>
-      <c r="C44" s="4" t="s">
+      <c r="D44" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B45" s="18"/>
+      <c r="C45" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="D44" t="s">
+      <c r="D45" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B45" s="13"/>
-      <c r="C45" s="4" t="s">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B46" s="18"/>
+      <c r="C46" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="D45" t="s">
+      <c r="D46" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B46" s="13"/>
-      <c r="C46" s="4" t="s">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B47" s="18"/>
+      <c r="C47" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="D46" t="s">
+      <c r="D47" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B47" t="s">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B48" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="C47" s="4" t="s">
+      <c r="C48" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="D47" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C48" s="4" t="s">
+      <c r="D48" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B49" s="18"/>
+      <c r="C49" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="D48" t="s">
+      <c r="D49" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A50" s="2" t="s">
+      <c r="B50" t="s">
+        <v>85</v>
+      </c>
+      <c r="C50" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="D50" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A52" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="B51" s="3" t="s">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B53" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C51" s="3" t="s">
+      <c r="C53" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D51" t="s">
+      <c r="D53" t="s">
         <v>32</v>
       </c>
-      <c r="E51" t="s">
+      <c r="E53" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="B52" s="9" t="s">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B54" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="C52" s="6" t="s">
+      <c r="C54" s="6" t="s">
         <v>23</v>
-      </c>
-      <c r="D52">
-        <v>4</v>
-      </c>
-      <c r="E52">
-        <f>SUM(D52:D65)</f>
-        <v>44</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="B53" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="C53" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D53">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="B54" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="C54" s="6" t="s">
-        <v>24</v>
       </c>
       <c r="D54">
         <v>4</v>
       </c>
+      <c r="E54">
+        <f>SUM(D54:D67)</f>
+        <v>44</v>
+      </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="B55" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="C55" s="7" t="s">
-        <v>25</v>
+      <c r="B55" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>31</v>
       </c>
       <c r="D55">
         <v>4</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="B56" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="C56" s="7" t="s">
-        <v>26</v>
+      <c r="B56" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>24</v>
       </c>
       <c r="D56">
         <v>4</v>
@@ -1120,43 +1135,43 @@
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B57" s="11" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D57">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B58" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="C58" s="7">
-        <v>1</v>
+        <v>12</v>
+      </c>
+      <c r="C58" s="7" t="s">
+        <v>26</v>
       </c>
       <c r="D58">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B59" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="C59" s="7">
-        <v>48000</v>
+        <v>13</v>
+      </c>
+      <c r="C59" s="7" t="s">
+        <v>27</v>
       </c>
       <c r="D59">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B60" s="11" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C60" s="7">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D60">
         <v>2</v>
@@ -1164,10 +1179,10 @@
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B61" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="C61" s="7" t="s">
-        <v>29</v>
+        <v>15</v>
+      </c>
+      <c r="C61" s="7">
+        <v>48000</v>
       </c>
       <c r="D61">
         <v>4</v>
@@ -1175,101 +1190,125 @@
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B62" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="C62" s="7" t="s">
-        <v>30</v>
+        <v>18</v>
+      </c>
+      <c r="C62" s="7">
+        <v>16</v>
       </c>
       <c r="D62">
         <v>2</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="B63" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="C63" s="8" t="s">
-        <v>28</v>
+      <c r="B63" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C63" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="D63">
         <v>4</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="B64" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="C64" s="8" t="s">
-        <v>35</v>
+      <c r="B64" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C64" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D64">
+        <v>2</v>
       </c>
     </row>
     <row r="65" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B65" s="8" t="s">
-        <v>20</v>
+      <c r="B65" s="12" t="s">
+        <v>19</v>
       </c>
       <c r="C65" s="8" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="D65">
         <v>4</v>
       </c>
     </row>
     <row r="66" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B66" s="8" t="s">
+      <c r="B66" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="C66" s="8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="67" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B67" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C67" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D67">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="68" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B68" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C66" s="8" t="s">
+      <c r="C68" s="8" t="s">
         <v>36</v>
-      </c>
-    </row>
-    <row r="67" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B67" t="s">
-        <v>42</v>
-      </c>
-      <c r="C67" s="16" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="68" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B68" t="s">
-        <v>73</v>
-      </c>
-      <c r="C68" s="16" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="69" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B69" t="s">
-        <v>75</v>
+        <v>42</v>
       </c>
       <c r="C69" s="16" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
     </row>
     <row r="70" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B70" t="s">
+        <v>73</v>
+      </c>
+      <c r="C70" s="16" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="71" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B71" t="s">
+        <v>75</v>
+      </c>
+      <c r="C71" s="16" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="72" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B72" t="s">
         <v>77</v>
       </c>
-      <c r="C70" s="16" t="s">
+      <c r="C72" s="16" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="71" spans="2:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="B71" t="s">
+    <row r="73" spans="2:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="B73" t="s">
         <v>79</v>
       </c>
-      <c r="C71" s="18" t="s">
+      <c r="C73" s="17" t="s">
         <v>80</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="B43:B46"/>
+  <mergeCells count="8">
+    <mergeCell ref="B48:B49"/>
+    <mergeCell ref="B44:B47"/>
     <mergeCell ref="C11:C24"/>
-    <mergeCell ref="C40:C42"/>
+    <mergeCell ref="C41:C43"/>
     <mergeCell ref="B10:B26"/>
-    <mergeCell ref="B36:B42"/>
+    <mergeCell ref="B37:B43"/>
     <mergeCell ref="B27:B30"/>
+    <mergeCell ref="B31:B32"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>